<commit_message>
Agrega salas y mejora reservas y seguridad
</commit_message>
<xml_diff>
--- a/plantillas/plantilla_ocupacion_aulas.xlsx
+++ b/plantillas/plantilla_ocupacion_aulas.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ocupación" sheetId="1" r:id="Rcdc270576eb548d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R846ad46a8dcc4cff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ocupación" sheetId="1" r:id="R8a96025eff9845f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Rf3d18e29bb834798"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3057,7 +3057,7 @@
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="A2:A201">
-      <x:formula1>"L601,L602,L603,708,709,710,711"</x:formula1>
+      <x:formula1>"L601,L602,L603,708,709,710,711,SS-3P,SR-1P"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="B2:B201">
       <x:formula1>"LUNES,MARTES,MIÉRCOLES,JUEVES,VIERNES,SÁBADO"</x:formula1>
@@ -3068,7 +3068,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34e9ae3532ae4763"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a114c5b651d49ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3115,7 +3115,7 @@
         <x:v>Aula</x:v>
       </x:c>
       <x:c r="B5" s="47" t="str">
-        <x:v>Seleccione L601, L602, L603, 708, 709, 710 o 711.</x:v>
+        <x:v>Seleccione L601, L602, L603, 708, 709, 710, 711, SS-3P o SR-1P.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="32" customHeight="1">
@@ -3204,7 +3204,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b200bf6f5f945bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9892af0856d64b91"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>